<commit_message>
Regenerate the 2026-27 and later packages and their reconciliation reports at 55p
Packages: SE, BST and Taxi 2027-04-05, and every Company year end mapped to
ltd-2026 or ltd-2027. Reports: the Apr27 SE, BST and Taxi scenarios and the
Company scenario-full at Mar27 and Oct27; all reconcile.

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Model: claude-sonnet-5-5
Claude-Session: https://claude.ai/code/session_01VyobNtzoueeNnQKC2bkP4e
</commit_message>
<xml_diff>
--- a/packages/GB Accounts Company 2026-04-30 (Apr26) Excel 2007/Financialaccounts.xlsx
+++ b/packages/GB Accounts Company 2026-04-30 (Apr26) Excel 2007/Financialaccounts.xlsx
@@ -16797,7 +16797,7 @@
         <v>10000</v>
       </c>
       <c r="O16" s="266">
-        <v>0.45</v>
+        <v>0.55</v>
       </c>
       <c r="P16" s="253"/>
       <c r="Q16" s="253"/>
@@ -30694,7 +30694,7 @@
       </c>
       <c r="EG58" s="13"/>
       <c r="EH58" s="22">
-        <f>IF(OpenAccounts!P8="X",0,EF58/((100-Admin!P7)/100)-EF58)</f>
+        <f>ROUND(IF(OpenAccounts!P8="X",0,EF58/((100-Admin!P7)/100)-EF58),2)</f>
         <v>0</v>
       </c>
       <c r="EI58" s="13"/>
@@ -45203,7 +45203,7 @@
       <c r="I35" s="188"/>
       <c r="J35" s="188"/>
       <c r="K35" s="189">
-        <f>SUM(I33:I34)</f>
+        <f>ROUND(SUM(I33:I34),2)</f>
         <v>0</v>
       </c>
       <c r="L35" s="39"/>
@@ -53434,7 +53434,7 @@
       </c>
       <c r="X135" s="225"/>
       <c r="Y135" s="535">
-        <f>AJ131-Y133</f>
+        <f>CorporationTax!K35</f>
         <v>0</v>
       </c>
       <c r="Z135" s="535"/>

</xml_diff>